<commit_message>
Updated field names in order to merge.
</commit_message>
<xml_diff>
--- a/Median_Final.xlsx
+++ b/Median_Final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R Projects\demographics-arcgis-hub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E005150-0026-4C6A-B211-498E3BCFDB3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8A59579-9857-4FB8-A02D-F8F8BC0D1A58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{2F75E0D1-E0F4-4592-A1BA-53D68C26F0CC}"/>
   </bookViews>
@@ -25,16 +25,16 @@
     <t>CouncilDistrict</t>
   </si>
   <si>
-    <t>MedianHouseholdIncome</t>
+    <t>MedianCommute</t>
   </si>
   <si>
-    <t>MedianFamilyIncome</t>
+    <t>MedianAgeE</t>
   </si>
   <si>
-    <t>MedianAge</t>
+    <t>MedianFamilyIncomeE</t>
   </si>
   <si>
-    <t>MedianCommute</t>
+    <t>MedianHouseholdIncomeE</t>
   </si>
 </sst>
 </file>
@@ -903,16 +903,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>